<commit_message>
20260506: updated updates-qmds files for GMACS updates through 20250505
</commit_message>
<xml_diff>
--- a/updates-qmds/Updates_Tables.xlsx
+++ b/updates-qmds/Updates_Tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamstockhausen/Work/Programming/GMACS-project/GMACS_tpl-cpp_code/updates-qmds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE0B48C4-9AFD-E848-8A15-436CD40F4D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862C4F95-C77A-ED4A-B700-A212EC17ACA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1880" windowWidth="38400" windowHeight="18380" activeTab="1" xr2:uid="{26300152-2BE3-3743-8659-A705683371A8}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="148">
   <si>
     <t>AEP</t>
   </si>
@@ -627,6 +627,32 @@
   </si>
   <si>
     <t>Added NO_PRIOR (= -1) as possible prior for parameters. Sets the prior_pdf = 0 for the term in question(perhaps simpler than using UNIFORM_PRIOR (= 0)).</t>
+  </si>
+  <si>
+    <t>2.20.37</t>
+  </si>
+  <si>
+    <t>devel_202605</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Added new options for calculating/extending size comps and modified output/input files to reflect new options. Added CATCH_COMP_NOSCL (=-1) and renamed CATCH_COMP (=1) to CATCH_COMP_DOSCL to provide sample size scaling/no scaling options for input fishery size comps. Added SURVEY_COMP_NOSCL (=-2) and renamed SURVEY_COMP (=2) to SURVEY_COMP_DOSCL to provide sample size scaling/no scaling options for input survey size comps.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Fixed calculation of predicted fishery size comps in calc_predicted_composition by including fully-selected F's (ft(k,h,i,j)) in the calculations. Calculation of predicted survey size comps in calc_predicted_composition *should* be correct because the calculations apply appropriate q's to the predicted comps. Reformatted some sections of code for better(?) readability.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1897,7 +1923,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{759BE828-8905-E144-8449-D0ED6D872523}">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.33203125" style="5" customWidth="1"/>
@@ -2362,6 +2388,23 @@
         <v>131</v>
       </c>
     </row>
+    <row r="30" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+      <c r="A30" s="4">
+        <v>46147</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.3" footer="0.3"/>
   <pageSetup scale="50" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
20260507. Changed Derived_quatities to Derived_quantities in gmacs.rep1 file. Updated Updates_Tables files.
</commit_message>
<xml_diff>
--- a/updates-qmds/Updates_Tables.xlsx
+++ b/updates-qmds/Updates_Tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamstockhausen/Work/Programming/GMACS-project/GMACS_tpl-cpp_code/updates-qmds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862C4F95-C77A-ED4A-B700-A212EC17ACA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FBA8CE8-B69A-B74A-A7FD-4B9DD69E728D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1880" windowWidth="38400" windowHeight="18380" activeTab="1" xr2:uid="{26300152-2BE3-3743-8659-A705683371A8}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="150">
   <si>
     <t>AEP</t>
   </si>
@@ -653,6 +653,12 @@
       </rPr>
       <t xml:space="preserve"> Fixed calculation of predicted fishery size comps in calc_predicted_composition by including fully-selected F's (ft(k,h,i,j)) in the calculations. Calculation of predicted survey size comps in calc_predicted_composition *should* be correct because the calculations apply appropriate q's to the predicted comps. Reformatted some sections of code for better(?) readability.</t>
     </r>
+  </si>
+  <si>
+    <t>Added checks on `hasMMOD` for calculations and output wrto male maturity ogive data. Fixed error when trying to normalize a predicted size comp with all 0's. Added origCol and aggCol to Size_fit_summary dataframe in gmacs.rep1.</t>
+  </si>
+  <si>
+    <t>Changed "Derived_quatities" to "Derived_quantities" in gmacs.rep1. Updated compile date.</t>
   </si>
 </sst>
 </file>
@@ -1923,10 +1929,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{759BE828-8905-E144-8449-D0ED6D872523}">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" style="4" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="6"/>
     <col min="3" max="3" width="10.83203125" style="5"/>
     <col min="4" max="4" width="89.6640625" style="8" customWidth="1"/>
@@ -2392,7 +2398,7 @@
       <c r="A30" s="4">
         <v>46147</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C30" s="5" t="s">
@@ -2404,6 +2410,295 @@
       <c r="E30" s="5" t="s">
         <v>146</v>
       </c>
+    </row>
+    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="A31" s="4">
+        <v>46148</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A32" s="4">
+        <v>46149</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B33" s="5"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B34" s="5"/>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B35" s="5"/>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B36" s="5"/>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B37" s="5"/>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B38" s="5"/>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B39" s="5"/>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B40" s="5"/>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B41" s="5"/>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B42" s="5"/>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B43" s="5"/>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B44" s="5"/>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B45" s="5"/>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B46" s="5"/>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B47" s="5"/>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B48" s="5"/>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B49" s="5"/>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B50" s="5"/>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B51" s="5"/>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B52" s="5"/>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B53" s="5"/>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B54" s="5"/>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B55" s="5"/>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B56" s="5"/>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B57" s="5"/>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B58" s="5"/>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B59" s="5"/>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B60" s="5"/>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B61" s="5"/>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B62" s="5"/>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B63" s="5"/>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B64" s="5"/>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B65" s="5"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B66" s="5"/>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B67" s="5"/>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B68" s="5"/>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B69" s="5"/>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B70" s="5"/>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B71" s="5"/>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B72" s="5"/>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B73" s="5"/>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B74" s="5"/>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B75" s="5"/>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B76" s="5"/>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B77" s="5"/>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B78" s="5"/>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B79" s="5"/>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B80" s="5"/>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B81" s="5"/>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B82" s="5"/>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B83" s="5"/>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B84" s="5"/>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B85" s="5"/>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B86" s="5"/>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B87" s="5"/>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B88" s="5"/>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B89" s="5"/>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B90" s="5"/>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B91" s="5"/>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B92" s="5"/>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B93" s="5"/>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B94" s="5"/>
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B95" s="5"/>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B96" s="5"/>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B97" s="5"/>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B98" s="5"/>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B99" s="5"/>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B100" s="5"/>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B101" s="5"/>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B102" s="5"/>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B103" s="5"/>
+    </row>
+    <row r="104" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B104" s="5"/>
+    </row>
+    <row r="105" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B105" s="5"/>
+    </row>
+    <row r="106" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B106" s="5"/>
+    </row>
+    <row r="107" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B107" s="5"/>
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B108" s="5"/>
+    </row>
+    <row r="109" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B109" s="5"/>
+    </row>
+    <row r="110" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B110" s="5"/>
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B111" s="5"/>
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B112" s="5"/>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B113" s="5"/>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B114" s="5"/>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B115" s="5"/>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B116" s="5"/>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B117" s="5"/>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B118" s="5"/>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B119" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.3" footer="0.3"/>

</xml_diff>